<commit_message>
Improve image generation, LoRA training, and studio UX
</commit_message>
<xml_diff>
--- a/Excel/String.xlsx
+++ b/Excel/String.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" r:id="R2358f7c912aa49df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Define" sheetId="2" r:id="Rc55efde186494c8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" r:id="Rde2c5120e3614fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Define" sheetId="2" r:id="R6a1d7bcc80ba4528"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12282,10 +12282,10 @@
         <x:v>EidolonText117</x:v>
       </x:c>
       <x:c r="C614" s="3" t="str">
-        <x:v>선택한 모델과 같은 계열의 LoRA를 적용합니다.</x:v>
+        <x:v>같은 계열의 LoRA를 여러 개 선택할 수 있습니다. 저장된 트리거는 생성 프롬프트에 자동 적용됩니다.</x:v>
       </x:c>
       <x:c r="D614" s="3" t="str">
-        <x:v>Apply LoRAs from the same family as the selected model.</x:v>
+        <x:v>Select multiple LoRAs from the same model family. Their saved triggers are automatically applied to the generation prompt.</x:v>
       </x:c>
     </x:row>
     <x:row r="615" ht="16.5" hidden="0" customHeight="1">
@@ -12352,10 +12352,10 @@
         <x:v>EidolonText122</x:v>
       </x:c>
       <x:c r="C619" s="3" t="str">
-        <x:v>이미지 저장</x:v>
+        <x:v>다른 이름으로 저장</x:v>
       </x:c>
       <x:c r="D619" s="3" t="str">
-        <x:v>Save image</x:v>
+        <x:v>Save a copy</x:v>
       </x:c>
     </x:row>
     <x:row r="620" ht="16.5" hidden="0" customHeight="1">
@@ -12604,10 +12604,10 @@
         <x:v>EidolonText140</x:v>
       </x:c>
       <x:c r="C637" s="3" t="str">
-        <x:v>이미지 폴더</x:v>
+        <x:v>학습할 이미지</x:v>
       </x:c>
       <x:c r="D637" s="3" t="str">
-        <x:v>Image folder</x:v>
+        <x:v>Training images</x:v>
       </x:c>
     </x:row>
     <x:row r="638" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -12632,10 +12632,10 @@
         <x:v>EidolonText142</x:v>
       </x:c>
       <x:c r="C639" s="3" t="str">
-        <x:v>선택</x:v>
+        <x:v>폴더 선택</x:v>
       </x:c>
       <x:c r="D639" s="3" t="str">
-        <x:v>Browse</x:v>
+        <x:v>Choose folder</x:v>
       </x:c>
     </x:row>
     <x:row r="640" ht="16.5" hidden="0" customHeight="1">
@@ -12758,10 +12758,10 @@
         <x:v>EidolonText151</x:v>
       </x:c>
       <x:c r="C648" s="3" t="str">
-        <x:v>작업 폴더에서 학습 로그와 결과 가중치를 확인할 수 있습니다.</x:v>
+        <x:v>완료·실패·취소한 학습을 확인합니다. 학습한 LoRA는 생성 화면에서 선택해 사용할 수 있습니다.</x:v>
       </x:c>
       <x:c r="D648" s="3" t="str">
-        <x:v>Open a job folder to find its training log and output weights.</x:v>
+        <x:v>Review completed, failed or cancelled training. Select a trained LoRA in Generate to use it.</x:v>
       </x:c>
     </x:row>
     <x:row r="649" ht="16.5" hidden="0" customHeight="1">
@@ -13136,10 +13136,10 @@
         <x:v>EidolonText178</x:v>
       </x:c>
       <x:c r="C675" s="3" t="str">
-        <x:v>긍정 프롬프트</x:v>
+        <x:v>공용 긍정 프롬프트</x:v>
       </x:c>
       <x:c r="D675" s="3" t="str">
-        <x:v>Positive prompt</x:v>
+        <x:v>Shared positive prompt</x:v>
       </x:c>
     </x:row>
     <x:row r="676" ht="16.5" hidden="0" customHeight="1">
@@ -13164,10 +13164,10 @@
         <x:v>EidolonText180</x:v>
       </x:c>
       <x:c r="C677" s="3" t="str">
-        <x:v>부정 프롬프트</x:v>
+        <x:v>공용 부정 프롬프트</x:v>
       </x:c>
       <x:c r="D677" s="3" t="str">
-        <x:v>Negative prompt</x:v>
+        <x:v>Shared negative prompt</x:v>
       </x:c>
     </x:row>
     <x:row r="678" ht="16.5" hidden="0" customHeight="1">
@@ -13262,10 +13262,10 @@
         <x:v>EidolonText187</x:v>
       </x:c>
       <x:c r="C684" s="3" t="str">
-        <x:v>기본 SDXL Base 1.0 모델 다운로드를 선택하거나 모델·LoRA 탭에서 .safetensors 파일을 가져옵니다. 설치된 모델만 표시하며 SDXL을 기본으로 선택합니다. 최초 설치에는 인터넷 연결과 여러 GB의 여유 공간이 필요합니다.</x:v>
+        <x:v>기본 SDXL Base 1.0 모델 다운로드를 선택하거나 엔진의 모델·LoRA 탭에서 .safetensors 파일을 가져옵니다. 설치된 모델만 표시하며 SDXL을 기본으로 선택합니다. 최초 설치에는 인터넷 연결과 여러 GB의 여유 공간이 필요합니다.</x:v>
       </x:c>
       <x:c r="D684" s="3" t="str">
-        <x:v>Download the default SDXL Base 1.0 model, or import a .safetensors file in Models and LoRAs. Only installed models are shown, with SDXL selected by default. Initial setup requires internet access and several GB of free space.</x:v>
+        <x:v>Download the default SDXL Base 1.0 model, or import a .safetensors file in Engine &gt; Models and LoRAs. Only installed models are shown, with SDXL selected by default. Initial setup requires internet access and several GB of free space.</x:v>
       </x:c>
     </x:row>
     <x:row r="685" ht="16.5" hidden="0" customHeight="1">
@@ -13276,10 +13276,10 @@
         <x:v>EidolonText188</x:v>
       </x:c>
       <x:c r="C685" s="3" t="str">
-        <x:v>엔진 탭에는 ComfyUI 서버 주소만 입력합니다. 실행 중인 서버가 있으면 연결하고 로컬 주소에 서버가 없으면 설치한 엔진을 실행합니다. 앱이 시작한 서버는 종료 시 함께 종료하며 기존 서버는 유지합니다.</x:v>
+        <x:v>프롬프트로 이미지 생성</x:v>
       </x:c>
       <x:c r="D685" s="3" t="str">
-        <x:v>Enter the ComfyUI server address in Engine. Connect to an existing server, or start the installed engine if no server is running at a local address. Servers started by this app stop when it closes; existing servers keep running.</x:v>
+        <x:v>Generate from a prompt</x:v>
       </x:c>
     </x:row>
     <x:row r="686" ht="105.5999984741211" hidden="0" customHeight="1">
@@ -13290,10 +13290,10 @@
         <x:v>EidolonText189</x:v>
       </x:c>
       <x:c r="C686" s="3" t="str">
-        <x:v>생성 탭에서 만들고 싶은 장면을 입력하고 대기열에 추가를 누릅니다. 설치된 모델만 선택 목록에 표시합니다. 기본 모델을 선택한 뒤에는 프롬프트만 입력하면 됩니다. 실행 중에도 다음 요청을 추가할 수 있습니다.</x:v>
+        <x:v>생성 탭에서 만들고 싶은 장면을 입력하고 대기열에 추가를 누릅니다. 설치된 모델만 선택 목록에 표시합니다. 배경 투명하게를 체크하면 최종 이미지를 투명 PNG로 저장합니다. 실행 중에도 다음 요청을 추가할 수 있습니다.</x:v>
       </x:c>
       <x:c r="D686" s="3" t="str">
-        <x:v>In Generate, describe your scene and press Add to queue. Only installed models appear in the selector. After choosing a default model, enter just a prompt. You can add more requests while a job is running.</x:v>
+        <x:v>In Generate, describe your scene and press Add to queue. Only installed models appear in the selector. Enable Transparent background to save the final image as a transparent PNG. You can add more requests while a job is running.</x:v>
       </x:c>
     </x:row>
     <x:row r="687" ht="105.5999984741211" hidden="0" customHeight="1">
@@ -13304,10 +13304,10 @@
         <x:v>EidolonText190</x:v>
       </x:c>
       <x:c r="C687" s="3" t="str">
-        <x:v>설정의 공용 긍정 프롬프트에는 반복할 스타일을, 부정 프롬프트에는 피할 표현을 입력하세요. 저장한 내용은 이후 생성에 적용됩니다. 생성 이력을 선택하면 프롬프트를 다시 사용할 수 있습니다.</x:v>
+        <x:v>설정의 공용 긍정 프롬프트에는 반복할 스타일을, 부정 프롬프트에는 피할 표현을 입력하세요. 저장한 내용은 생성 화면에도 표시되고 이후 생성에 적용됩니다. 생성 결과에서 프롬프트를 다시 사용할 수 있습니다.</x:v>
       </x:c>
       <x:c r="D687" s="3" t="str">
-        <x:v>Use the shared positive prompt in Settings for recurring styles, and the negative prompt for things to avoid. Saved prompts apply to later generations. Select a generation history entry to reuse its prompt.</x:v>
+        <x:v>Use the shared positive prompt in Settings for recurring styles, and the negative prompt for things to avoid. Saved prompts are shown in Generate and apply to later generations. Reuse a prompt from Results.</x:v>
       </x:c>
     </x:row>
     <x:row r="688" ht="16.5" hidden="0" customHeight="1">
@@ -13332,10 +13332,10 @@
         <x:v>EidolonText192</x:v>
       </x:c>
       <x:c r="C689" s="3" t="str">
-        <x:v>LoRA 학습 탭에서 기반 모델, 이미지 폴더, 이름과 트리거를 지정하고 대기열에 추가를 누릅니다. PNG·JPG·BMP와 하위 폴더, 같은 이름의 .txt 캡션을 지원합니다. 기존 LoRA 이어 학습을 켜면 저장된 가중치와 rank부터 추가 학습합니다. optimizer와 스케줄은 새로 시작하며 결과는 새 LoRA로 저장합니다. 원본 이미지와 LoRA는 보존합니다.</x:v>
+        <x:v>모델, 이미지와 LoRA 이름·트리거를 지정합니다. 단계 수를 입력하거나 빠른·기본 학습을 선택한 뒤 대기열에 추가합니다. 요청 버튼 옆에서 학습을 취소할 수 있습니다. 하단에는 진행 상태와 예상 남은 시간을 표시합니다. 학습한 LoRA를 생성에서 선택하면 트리거가 자동 적용됩니다.</x:v>
       </x:c>
       <x:c r="D689" s="3" t="str">
-        <x:v>In LoRA training, select a base model and image folder, enter a name and trigger, then add to queue. PNG, JPG, BMP, subfolders and matching .txt captions are supported. Enable Continue training an existing LoRA to start from its weights and rank. The optimizer and schedule start fresh, and a new LoRA is saved. Original images and LoRAs are preserved.</x:v>
+        <x:v>Choose a model, images, LoRA name and trigger. Enter steps or use Quick or Standard, then queue training. Cancel beside the request button. The footer shows progress and estimated time remaining. Selecting a trained LoRA applies its trigger automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="690" ht="105.5999984741211" hidden="0" customHeight="1">
@@ -13374,10 +13374,10 @@
         <x:v>EidolonText195</x:v>
       </x:c>
       <x:c r="C692" s="3" t="str">
-        <x:v>창 하단에서 현재 상태, 진행률과 대기 건수를 확인합니다. 작업 취소는 실행 중인 요청만 취소하며 다음 요청은 계속 실행합니다. 대기 작업 비우기는 아직 시작하지 않은 요청을 취소합니다. 앱을 종료하면 실행 중인 작업과 대기 요청을 취소합니다. 다운로드가 중단되면 같은 경로에 설치·복구를 다시 실행하세요.</x:v>
+        <x:v>하단에는 상태·진행률·남은 시간과 대기 건수만 표시합니다. 학습 취소는 학습 요청 버튼 옆에 있습니다. 생성·학습 화면의 대기열 목록에서 아직 시작하지 않은 요청을 비울 수 있습니다. 앱 종료 시 실행 중인 작업과 대기 요청을 정리합니다.</x:v>
       </x:c>
       <x:c r="D692" s="3" t="str">
-        <x:v>Check the current status, progress and pending count at the bottom of the window. Cancel job cancels the running request and the next request continues. Clear pending jobs cancels requests that have not started. Closing the app cancels running and pending requests. If a download stops, run install or repair at the same path.</x:v>
+        <x:v>The footer displays status, progress, time remaining and pending count. Cancel training beside the request button. Clear requests that have not started from the queue in Generate or Train. Closing the app cleans up running and pending work.</x:v>
       </x:c>
     </x:row>
     <x:row r="693" ht="118.80000305175781" hidden="0" customHeight="1">
@@ -13684,14 +13684,14 @@
       <x:c r="C714" s="3" t="str">
         <x:v>
 {0} × {1} · seed {2}
-긍정: {3}
-부정: {4}</x:v>
+생성에 사용된 프롬프트: {3}
+부정 프롬프트: {4}</x:v>
       </x:c>
       <x:c r="D714" s="3" t="str">
         <x:v>
 {0} × {1} · seed {2}
-Positive: {3}
-Negative: {4}</x:v>
+Prompt used for generation: {3}
+Negative prompt: {4}</x:v>
       </x:c>
     </x:row>
     <x:row r="715" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -14450,6 +14450,1000 @@
       </x:c>
       <x:c r="D768" s="3" t="str">
         <x:v>Connect to server</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="769" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A769" s="2" t="n">
+        <x:v>3352</x:v>
+      </x:c>
+      <x:c r="B769" s="2" t="str">
+        <x:v>EidolonText272</x:v>
+      </x:c>
+      <x:c r="C769" s="3" t="str">
+        <x:v>설치된 엔진 모듈</x:v>
+      </x:c>
+      <x:c r="D769" s="3" t="str">
+        <x:v>Installed engine modules</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="770" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A770" s="2" t="n">
+        <x:v>3353</x:v>
+      </x:c>
+      <x:c r="B770" s="2" t="str">
+        <x:v>EidolonText273</x:v>
+      </x:c>
+      <x:c r="C770" s="3" t="str">
+        <x:v>목록 새로고침</x:v>
+      </x:c>
+      <x:c r="D770" s="3" t="str">
+        <x:v>Refresh list</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="771" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A771" s="2" t="n">
+        <x:v>3354</x:v>
+      </x:c>
+      <x:c r="B771" s="2" t="str">
+        <x:v>EidolonText274</x:v>
+      </x:c>
+      <x:c r="C771" s="3" t="str">
+        <x:v>실행 구성요소</x:v>
+      </x:c>
+      <x:c r="D771" s="3" t="str">
+        <x:v>Runtime components</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="772" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A772" s="2" t="n">
+        <x:v>3355</x:v>
+      </x:c>
+      <x:c r="B772" s="2" t="str">
+        <x:v>EidolonText275</x:v>
+      </x:c>
+      <x:c r="C772" s="3" t="str">
+        <x:v>ComfyUI 커스텀 노드</x:v>
+      </x:c>
+      <x:c r="D772" s="3" t="str">
+        <x:v>ComfyUI custom nodes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="773" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A773" s="2" t="n">
+        <x:v>3356</x:v>
+      </x:c>
+      <x:c r="B773" s="2" t="str">
+        <x:v>EidolonText276</x:v>
+      </x:c>
+      <x:c r="C773" s="3" t="str">
+        <x:v>설치됨</x:v>
+      </x:c>
+      <x:c r="D773" s="3" t="str">
+        <x:v>Installed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="774" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A774" s="2" t="n">
+        <x:v>3357</x:v>
+      </x:c>
+      <x:c r="B774" s="2" t="str">
+        <x:v>EidolonText277</x:v>
+      </x:c>
+      <x:c r="C774" s="3" t="str">
+        <x:v>미설치</x:v>
+      </x:c>
+      <x:c r="D774" s="3" t="str">
+        <x:v>Not installed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="775" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A775" s="2" t="n">
+        <x:v>3358</x:v>
+      </x:c>
+      <x:c r="B775" s="2" t="str">
+        <x:v>EidolonText278</x:v>
+      </x:c>
+      <x:c r="C775" s="3" t="str">
+        <x:v>비활성화</x:v>
+      </x:c>
+      <x:c r="D775" s="3" t="str">
+        <x:v>Disabled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="776" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A776" s="2" t="n">
+        <x:v>3359</x:v>
+      </x:c>
+      <x:c r="B776" s="2" t="str">
+        <x:v>EidolonText279</x:v>
+      </x:c>
+      <x:c r="C776" s="3" t="str">
+        <x:v>버전 정보 없음</x:v>
+      </x:c>
+      <x:c r="D776" s="3" t="str">
+        <x:v>Version unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="777" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A777" s="2" t="n">
+        <x:v>3360</x:v>
+      </x:c>
+      <x:c r="B777" s="2" t="str">
+        <x:v>EidolonText280</x:v>
+      </x:c>
+      <x:c r="C777" s="3" t="str">
+        <x:v>설치 경로를 선택하면 구성요소를 표시합니다.</x:v>
+      </x:c>
+      <x:c r="D777" s="3" t="str">
+        <x:v>Choose an installation path to view its components.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="778" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A778" s="2" t="n">
+        <x:v>3361</x:v>
+      </x:c>
+      <x:c r="B778" s="2" t="str">
+        <x:v>EidolonText281</x:v>
+      </x:c>
+      <x:c r="C778" s="3" t="str">
+        <x:v>설치된 커스텀 노드가 없습니다.</x:v>
+      </x:c>
+      <x:c r="D778" s="3" t="str">
+        <x:v>No installed custom nodes were found.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="779" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A779" s="2" t="n">
+        <x:v>3362</x:v>
+      </x:c>
+      <x:c r="B779" s="2" t="str">
+        <x:v>EidolonText282</x:v>
+      </x:c>
+      <x:c r="C779" s="3" t="str">
+        <x:v>Python (이미지 생성)</x:v>
+      </x:c>
+      <x:c r="D779" s="3" t="str">
+        <x:v>Python (generation)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="780" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A780" s="2" t="n">
+        <x:v>3363</x:v>
+      </x:c>
+      <x:c r="B780" s="2" t="str">
+        <x:v>EidolonText283</x:v>
+      </x:c>
+      <x:c r="C780" s="3" t="str">
+        <x:v>Python (LoRA 학습)</x:v>
+      </x:c>
+      <x:c r="D780" s="3" t="str">
+        <x:v>Python (LoRA training)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="781" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A781" s="2" t="n">
+        <x:v>3364</x:v>
+      </x:c>
+      <x:c r="B781" s="2" t="str">
+        <x:v>EidolonText284</x:v>
+      </x:c>
+      <x:c r="C781" s="3" t="str">
+        <x:v>선택한 로컬 설치 폴더의 구성요소와 커스텀 노드 파일을 표시합니다.</x:v>
+      </x:c>
+      <x:c r="D781" s="3" t="str">
+        <x:v>Show components and custom node files in the selected local installation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="782" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A782" s="2" t="n">
+        <x:v>3365</x:v>
+      </x:c>
+      <x:c r="B782" s="2" t="str">
+        <x:v>EidolonText285</x:v>
+      </x:c>
+      <x:c r="C782" s="3" t="str">
+        <x:v>엔진 탭에는 ComfyUI 서버 주소만 입력합니다. 실행 중인 서버가 있으면 연결하고 로컬 주소에 서버가 없으면 설치한 엔진을 실행합니다. 앱이 시작한 서버는 종료 시 함께 종료하며 기존 서버는 유지합니다.</x:v>
+      </x:c>
+      <x:c r="D782" s="3" t="str">
+        <x:v>Enter the ComfyUI server address in Engine. Connect to an existing server, or start the installed engine if no server is running at a local address. Servers started by this app stop when it closes; existing servers keep running.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="783" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A783" s="2" t="n">
+        <x:v>3366</x:v>
+      </x:c>
+      <x:c r="B783" s="2" t="str">
+        <x:v>EidolonText286</x:v>
+      </x:c>
+      <x:c r="C783" s="3" t="str">
+        <x:v>설치 목록을 불러오지 못했습니다. {0}</x:v>
+      </x:c>
+      <x:c r="D783" s="3" t="str">
+        <x:v>Could not load the installed modules. {0}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="784" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A784" s="2" t="n">
+        <x:v>3367</x:v>
+      </x:c>
+      <x:c r="B784" s="2" t="str">
+        <x:v>EidolonText287</x:v>
+      </x:c>
+      <x:c r="C784" s="3" t="str">
+        <x:v>기본 외곽선 추출 노드를 다운로드합니다.</x:v>
+      </x:c>
+      <x:c r="D784" s="3" t="str">
+        <x:v>Downloading the default outline extraction nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="785" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A785" s="2" t="n">
+        <x:v>3368</x:v>
+      </x:c>
+      <x:c r="B785" s="2" t="str">
+        <x:v>EidolonText288</x:v>
+      </x:c>
+      <x:c r="C785" s="3" t="str">
+        <x:v>외곽선 추출 노드의 실행 패키지를 설치합니다.</x:v>
+      </x:c>
+      <x:c r="D785" s="3" t="str">
+        <x:v>Installing dependencies for the outline extraction nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="786" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A786" s="2" t="n">
+        <x:v>3369</x:v>
+      </x:c>
+      <x:c r="B786" s="2" t="str">
+        <x:v>EidolonText289</x:v>
+      </x:c>
+      <x:c r="C786" s="3" t="str">
+        <x:v>커스텀 노드의 필수 파일이 없습니다. {0}</x:v>
+      </x:c>
+      <x:c r="D786" s="3" t="str">
+        <x:v>A required custom node file is missing. {0}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="787" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A787" s="2" t="n">
+        <x:v>3370</x:v>
+      </x:c>
+      <x:c r="B787" s="2" t="str">
+        <x:v>EidolonText290</x:v>
+      </x:c>
+      <x:c r="C787" s="3" t="str">
+        <x:v>외곽선 추출(Canny·Lineart) 노드도 기본 설치합니다. 기존 설치는 설치·복구를 실행해 추가하세요.</x:v>
+      </x:c>
+      <x:c r="D787" s="3" t="str">
+        <x:v>Canny and Lineart extraction nodes are installed by default. Run install or repair to add them to an existing installation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="788" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A788" s="2" t="n">
+        <x:v>3371</x:v>
+      </x:c>
+      <x:c r="B788" s="2" t="str">
+        <x:v>EidolonText291</x:v>
+      </x:c>
+      <x:c r="C788" s="3" t="str">
+        <x:v>생성 결과</x:v>
+      </x:c>
+      <x:c r="D788" s="3" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="789" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A789" s="2" t="n">
+        <x:v>3372</x:v>
+      </x:c>
+      <x:c r="B789" s="2" t="str">
+        <x:v>EidolonText292</x:v>
+      </x:c>
+      <x:c r="C789" s="3" t="str">
+        <x:v>입력 프롬프트</x:v>
+      </x:c>
+      <x:c r="D789" s="3" t="str">
+        <x:v>Input prompt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="790" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A790" s="2" t="n">
+        <x:v>3373</x:v>
+      </x:c>
+      <x:c r="B790" s="2" t="str">
+        <x:v>EidolonText293</x:v>
+      </x:c>
+      <x:c r="C790" s="3" t="str">
+        <x:v>실제 생성에 사용된 프롬프트</x:v>
+      </x:c>
+      <x:c r="D790" s="3" t="str">
+        <x:v>Prompt used for generation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="791" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A791" s="2" t="n">
+        <x:v>3374</x:v>
+      </x:c>
+      <x:c r="B791" s="2" t="str">
+        <x:v>EidolonText294</x:v>
+      </x:c>
+      <x:c r="C791" s="3" t="str">
+        <x:v>부정 프롬프트</x:v>
+      </x:c>
+      <x:c r="D791" s="3" t="str">
+        <x:v>Negative prompt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="792" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A792" s="2" t="n">
+        <x:v>3375</x:v>
+      </x:c>
+      <x:c r="B792" s="2" t="str">
+        <x:v>EidolonText295</x:v>
+      </x:c>
+      <x:c r="C792" s="3" t="str">
+        <x:v>이 결과로 학습</x:v>
+      </x:c>
+      <x:c r="D792" s="3" t="str">
+        <x:v>Use for training</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="793" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A793" s="2" t="n">
+        <x:v>3376</x:v>
+      </x:c>
+      <x:c r="B793" s="2" t="str">
+        <x:v>EidolonText296</x:v>
+      </x:c>
+      <x:c r="C793" s="3" t="str">
+        <x:v>이미지 폴더 열기</x:v>
+      </x:c>
+      <x:c r="D793" s="3" t="str">
+        <x:v>Open image folder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="794" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A794" s="2" t="n">
+        <x:v>3377</x:v>
+      </x:c>
+      <x:c r="B794" s="2" t="str">
+        <x:v>EidolonText297</x:v>
+      </x:c>
+      <x:c r="C794" s="3" t="str">
+        <x:v>생성 이미지 저장 폴더</x:v>
+      </x:c>
+      <x:c r="D794" s="3" t="str">
+        <x:v>Generated images folder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="795" ht="66" hidden="0" customHeight="1">
+      <x:c r="A795" s="2" t="n">
+        <x:v>3378</x:v>
+      </x:c>
+      <x:c r="B795" s="2" t="str">
+        <x:v>EidolonText298</x:v>
+      </x:c>
+      <x:c r="C795" s="3" t="str">
+        <x:v>새 생성의 최종 이미지만 이 폴더에 GUID.png로 저장합니다. 기본 경로는 사용자 AppData의 Eidolon\Images이며 다른 폴더를 지정할 수 있습니다. 원본은 Job 폴더에 보관하고 이전 결과는 이동하지 않습니다.</x:v>
+      </x:c>
+      <x:c r="D795" s="3" t="str">
+        <x:v>New generations save only the final image here as GUID.png. Default: Eidolon\Images under local AppData. You can choose another folder. Originals stay in job folders; previous results are not moved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="796" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A796" s="2" t="n">
+        <x:v>3379</x:v>
+      </x:c>
+      <x:c r="B796" s="2" t="str">
+        <x:v>EidolonText299</x:v>
+      </x:c>
+      <x:c r="C796" s="3" t="str">
+        <x:v>생성 이미지 저장 폴더 선택</x:v>
+      </x:c>
+      <x:c r="D796" s="3" t="str">
+        <x:v>Choose a folder for generated images</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="797" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A797" s="2" t="n">
+        <x:v>3380</x:v>
+      </x:c>
+      <x:c r="B797" s="2" t="str">
+        <x:v>EidolonText300</x:v>
+      </x:c>
+      <x:c r="C797" s="3" t="str">
+        <x:v>이미지 저장 폴더는 절대 경로를 입력하세요.</x:v>
+      </x:c>
+      <x:c r="D797" s="3" t="str">
+        <x:v>Enter an absolute path for the generated images folder.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="798" ht="66" hidden="0" customHeight="1">
+      <x:c r="A798" s="2" t="n">
+        <x:v>3381</x:v>
+      </x:c>
+      <x:c r="B798" s="2" t="str">
+        <x:v>EidolonText301</x:v>
+      </x:c>
+      <x:c r="C798" s="3" t="str">
+        <x:v>결과 이미지와 프롬프트를 가져왔습니다. 생성에 사용한 모델이 현재 목록에 없으므로 학습에 사용할 기반 모델을 선택하세요.</x:v>
+      </x:c>
+      <x:c r="D798" s="3" t="str">
+        <x:v>Loaded the result images and prompt. The model used for generation is not in the current list; select a base model for training.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="799" ht="66" hidden="0" customHeight="1">
+      <x:c r="A799" s="2" t="n">
+        <x:v>3382</x:v>
+      </x:c>
+      <x:c r="B799" s="2" t="str">
+        <x:v>EidolonText302</x:v>
+      </x:c>
+      <x:c r="C799" s="3" t="str">
+        <x:v>선택한 이미지와 생성에 사용된 프롬프트를 학습 입력으로 가져왔습니다. 이름과 트리거를 입력해 학습을 시작하세요.</x:v>
+      </x:c>
+      <x:c r="D799" s="3" t="str">
+        <x:v>Loaded the selected image and prompt used for generation into the training inputs. Enter a name and trigger to start training.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="800" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A800" s="2" t="n">
+        <x:v>3383</x:v>
+      </x:c>
+      <x:c r="B800" s="2" t="str">
+        <x:v>EidolonText303</x:v>
+      </x:c>
+      <x:c r="C800" s="3" t="str">
+        <x:v>이전 이미지와 적용된 프롬프트는 생성 결과 탭에서 확인하세요.</x:v>
+      </x:c>
+      <x:c r="D800" s="3" t="str">
+        <x:v>View previous images and their applied prompts in Results.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="801" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A801" s="2" t="n">
+        <x:v>3384</x:v>
+      </x:c>
+      <x:c r="B801" s="2" t="str">
+        <x:v>EidolonText304</x:v>
+      </x:c>
+      <x:c r="C801" s="3" t="str">
+        <x:v>이미지를 생성하면 사용한 프롬프트와 함께 이곳에 기록됩니다.</x:v>
+      </x:c>
+      <x:c r="D801" s="3" t="str">
+        <x:v>Generated images appear here together with the prompts used.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="802" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A802" s="2" t="n">
+        <x:v>3385</x:v>
+      </x:c>
+      <x:c r="B802" s="2" t="str">
+        <x:v>EidolonText305</x:v>
+      </x:c>
+      <x:c r="C802" s="3" t="str">
+        <x:v>이 결과로 학습은 선택한 이미지 한 장과 생성에 사용된 프롬프트를 학습 입력으로 가져옵니다. 이름·트리거와 이어 학습할 LoRA는 학습 탭에서 지정하세요.</x:v>
+      </x:c>
+      <x:c r="D802" s="3" t="str">
+        <x:v>Use for training fills the selected image and prompt used for generation. In Training, enter a name and trigger, and select a LoRA to continue training.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="803" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A803" s="2" t="n">
+        <x:v>3386</x:v>
+      </x:c>
+      <x:c r="B803" s="2" t="str">
+        <x:v>EidolonText306</x:v>
+      </x:c>
+      <x:c r="C803" s="3" t="str">
+        <x:v>사용된 모델</x:v>
+      </x:c>
+      <x:c r="D803" s="3" t="str">
+        <x:v>Model used</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="804" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A804" s="2" t="n">
+        <x:v>3387</x:v>
+      </x:c>
+      <x:c r="B804" s="2" t="str">
+        <x:v>EidolonText307</x:v>
+      </x:c>
+      <x:c r="C804" s="3" t="str">
+        <x:v>표시할 결과 이미지가 없습니다.</x:v>
+      </x:c>
+      <x:c r="D804" s="3" t="str">
+        <x:v>No result image to display.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="805" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A805" s="2" t="n">
+        <x:v>3388</x:v>
+      </x:c>
+      <x:c r="B805" s="2" t="str">
+        <x:v>EidolonText308</x:v>
+      </x:c>
+      <x:c r="C805" s="3" t="str">
+        <x:v>배경 투명하게</x:v>
+      </x:c>
+      <x:c r="D805" s="3" t="str">
+        <x:v>Transparent background</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="806" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A806" s="2" t="n">
+        <x:v>3389</x:v>
+      </x:c>
+      <x:c r="B806" s="2" t="str">
+        <x:v>EidolonText309</x:v>
+      </x:c>
+      <x:c r="C806" s="3" t="str">
+        <x:v>생성 후 배경을 제거해 저장 폴더에 최종 PNG 한 장을 저장합니다. 원본은 앱의 작업 폴더에 보관하며 처음 사용할 때 배경 제거 모델을 내려받습니다.</x:v>
+      </x:c>
+      <x:c r="D806" s="3" t="str">
+        <x:v>Remove the background after generation and save one final PNG in the output folder. The original is kept in the app job folder, and the removal model is downloaded on first use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="807" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A807" s="2" t="n">
+        <x:v>3390</x:v>
+      </x:c>
+      <x:c r="B807" s="2" t="str">
+        <x:v>EidolonText310</x:v>
+      </x:c>
+      <x:c r="C807" s="3" t="str">
+        <x:v>배경 제거 모델을 준비합니다.</x:v>
+      </x:c>
+      <x:c r="D807" s="3" t="str">
+        <x:v>Preparing the background removal model.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="808" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A808" s="2" t="n">
+        <x:v>3391</x:v>
+      </x:c>
+      <x:c r="B808" s="2" t="str">
+        <x:v>EidolonText311</x:v>
+      </x:c>
+      <x:c r="C808" s="3" t="str">
+        <x:v>이미지 배경을 제거합니다.</x:v>
+      </x:c>
+      <x:c r="D808" s="3" t="str">
+        <x:v>Removing the image background.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="809" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A809" s="2" t="n">
+        <x:v>3392</x:v>
+      </x:c>
+      <x:c r="B809" s="2" t="str">
+        <x:v>EidolonText312</x:v>
+      </x:c>
+      <x:c r="C809" s="3" t="str">
+        <x:v>배경을 제거한 투명 PNG를 저장했습니다.</x:v>
+      </x:c>
+      <x:c r="D809" s="3" t="str">
+        <x:v>Saved a transparent PNG with the background removed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="810" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A810" s="2" t="n">
+        <x:v>3393</x:v>
+      </x:c>
+      <x:c r="B810" s="2" t="str">
+        <x:v>EidolonText313</x:v>
+      </x:c>
+      <x:c r="C810" s="3" t="str">
+        <x:v>선택한 생성 기록이나 이미지가 없습니다.</x:v>
+      </x:c>
+      <x:c r="D810" s="3" t="str">
+        <x:v>The selected generation record or image is unavailable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="811" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A811" s="2" t="n">
+        <x:v>3394</x:v>
+      </x:c>
+      <x:c r="B811" s="2" t="str">
+        <x:v>EidolonText314</x:v>
+      </x:c>
+      <x:c r="C811" s="3" t="str">
+        <x:v>실행 중인 생성 작업의 기록은 변경할 수 없습니다.</x:v>
+      </x:c>
+      <x:c r="D811" s="3" t="str">
+        <x:v>A running generation record cannot be changed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="812" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A812" s="2" t="n">
+        <x:v>3395</x:v>
+      </x:c>
+      <x:c r="B812" s="2" t="str">
+        <x:v>EidolonText315</x:v>
+      </x:c>
+      <x:c r="C812" s="3" t="str">
+        <x:v>이미지 배경을 제거하지 못했습니다. 로그를 확인하세요.</x:v>
+      </x:c>
+      <x:c r="D812" s="3" t="str">
+        <x:v>Could not remove the image background. Check the logs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="813" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A813" s="2" t="n">
+        <x:v>3396</x:v>
+      </x:c>
+      <x:c r="B813" s="2" t="str">
+        <x:v>EidolonText316</x:v>
+      </x:c>
+      <x:c r="C813" s="3" t="str">
+        <x:v>선택 삭제</x:v>
+      </x:c>
+      <x:c r="D813" s="3" t="str">
+        <x:v>Delete selected</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="814" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A814" s="2" t="n">
+        <x:v>3397</x:v>
+      </x:c>
+      <x:c r="B814" s="2" t="str">
+        <x:v>EidolonText317</x:v>
+      </x:c>
+      <x:c r="C814" s="3" t="str">
+        <x:v>전체 삭제</x:v>
+      </x:c>
+      <x:c r="D814" s="3" t="str">
+        <x:v>Delete all</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="815" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A815" s="2" t="n">
+        <x:v>3398</x:v>
+      </x:c>
+      <x:c r="B815" s="2" t="str">
+        <x:v>EidolonText318</x:v>
+      </x:c>
+      <x:c r="C815" s="3" t="str">
+        <x:v>생성 기록 삭제</x:v>
+      </x:c>
+      <x:c r="D815" s="3" t="str">
+        <x:v>Delete generation history</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="816" ht="66" hidden="0" customHeight="1">
+      <x:c r="A816" s="2" t="n">
+        <x:v>3399</x:v>
+      </x:c>
+      <x:c r="B816" s="2" t="str">
+        <x:v>EidolonText319</x:v>
+      </x:c>
+      <x:c r="C816" s="3" t="str">
+        <x:v>선택한 생성 기록과 Job 폴더를 삭제할까요? 프롬프트·모델 정보와 Job 폴더의 원본 이미지는 삭제됩니다. 최종 저장 이미지와 학습 기록은 보존합니다.</x:v>
+      </x:c>
+      <x:c r="D816" s="3" t="str">
+        <x:v>Delete the selected generation record and job folder? Prompt and model information and original images in the job folder will be removed. Final saved images and training records are kept.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="817" ht="66" hidden="0" customHeight="1">
+      <x:c r="A817" s="2" t="n">
+        <x:v>3400</x:v>
+      </x:c>
+      <x:c r="B817" s="2" t="str">
+        <x:v>EidolonText320</x:v>
+      </x:c>
+      <x:c r="C817" s="3" t="str">
+        <x:v>생성 기록 {0}개와 해당 Job 폴더를 모두 삭제할까요? 프롬프트·모델 정보와 원본 이미지는 삭제됩니다. 최종 저장 이미지와 학습 기록은 보존합니다.</x:v>
+      </x:c>
+      <x:c r="D817" s="3" t="str">
+        <x:v>Delete all {0} generation records and their job folders? Prompt and model information and original images will be removed. Final saved images and training records are kept.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="818" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A818" s="2" t="n">
+        <x:v>3401</x:v>
+      </x:c>
+      <x:c r="B818" s="2" t="str">
+        <x:v>EidolonText321</x:v>
+      </x:c>
+      <x:c r="C818" s="3" t="str">
+        <x:v>삭제</x:v>
+      </x:c>
+      <x:c r="D818" s="3" t="str">
+        <x:v>Delete</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="819" ht="16.5" hidden="0" customHeight="1">
+      <x:c r="A819" s="2" t="n">
+        <x:v>3402</x:v>
+      </x:c>
+      <x:c r="B819" s="2" t="str">
+        <x:v>EidolonText322</x:v>
+      </x:c>
+      <x:c r="C819" s="3" t="str">
+        <x:v>취소</x:v>
+      </x:c>
+      <x:c r="D819" s="3" t="str">
+        <x:v>Cancel</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="820" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A820" s="2" t="n">
+        <x:v>3403</x:v>
+      </x:c>
+      <x:c r="B820" s="2" t="str">
+        <x:v>EidolonText323</x:v>
+      </x:c>
+      <x:c r="C820" s="3" t="str">
+        <x:v>생성 기록 {0}개와 Job 폴더를 삭제했습니다. 최종 저장 이미지는 보존했습니다.</x:v>
+      </x:c>
+      <x:c r="D820" s="3" t="str">
+        <x:v>Deleted {0} generation records and their job folders. Final saved images were kept.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="821" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A821" s="2" t="n">
+        <x:v>3404</x:v>
+      </x:c>
+      <x:c r="B821" s="2" t="str">
+        <x:v>EidolonText324</x:v>
+      </x:c>
+      <x:c r="C821" s="3" t="str">
+        <x:v>표시된 결과 이미지 한 장만 학습합니다. 폴더 열기로 위치를 확인하거나 폴더로 변경을 눌러 폴더 전체를 학습할 수 있습니다.</x:v>
+      </x:c>
+      <x:c r="D821" s="3" t="str">
+        <x:v>Train only the result image shown here. Open folder shows its location. Use Switch to folder to train every image in a folder instead.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="822">
+      <x:c r="A822" s="2" t="n">
+        <x:v>3405</x:v>
+      </x:c>
+      <x:c r="B822" s="2" t="str">
+        <x:v>EidolonText325</x:v>
+      </x:c>
+      <x:c r="C822" s="3" t="str">
+        <x:v>아직 이미지가 없습니다</x:v>
+      </x:c>
+      <x:c r="D822" s="3" t="str">
+        <x:v>No images yet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="823">
+      <x:c r="A823" s="2" t="n">
+        <x:v>3406</x:v>
+      </x:c>
+      <x:c r="B823" s="2" t="str">
+        <x:v>EidolonText326</x:v>
+      </x:c>
+      <x:c r="C823" s="3" t="str">
+        <x:v>빠른 학습</x:v>
+      </x:c>
+      <x:c r="D823" s="3" t="str">
+        <x:v>Quick training</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="824">
+      <x:c r="A824" s="2" t="n">
+        <x:v>3407</x:v>
+      </x:c>
+      <x:c r="B824" s="2" t="str">
+        <x:v>EidolonText327</x:v>
+      </x:c>
+      <x:c r="C824" s="3" t="str">
+        <x:v>학습 취소</x:v>
+      </x:c>
+      <x:c r="D824" s="3" t="str">
+        <x:v>Cancel training</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="825">
+      <x:c r="A825" s="2" t="n">
+        <x:v>3408</x:v>
+      </x:c>
+      <x:c r="B825" s="2" t="str">
+        <x:v>EidolonText328</x:v>
+      </x:c>
+      <x:c r="C825" s="3" t="str">
+        <x:v>학습 취소 중…</x:v>
+      </x:c>
+      <x:c r="D825" s="3" t="str">
+        <x:v>Cancelling training…</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="826">
+      <x:c r="A826" s="2" t="n">
+        <x:v>3409</x:v>
+      </x:c>
+      <x:c r="B826" s="2" t="str">
+        <x:v>EidolonText329</x:v>
+      </x:c>
+      <x:c r="C826" s="3" t="str">
+        <x:v>예상 남은 시간: {0}</x:v>
+      </x:c>
+      <x:c r="D826" s="3" t="str">
+        <x:v>Estimated time remaining: {0}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="827">
+      <x:c r="A827" s="2" t="n">
+        <x:v>3410</x:v>
+      </x:c>
+      <x:c r="B827" s="2" t="str">
+        <x:v>EidolonText330</x:v>
+      </x:c>
+      <x:c r="C827" s="3" t="str">
+        <x:v>남은 시간 계산 중…</x:v>
+      </x:c>
+      <x:c r="D827" s="3" t="str">
+        <x:v>Estimating time remaining…</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="828">
+      <x:c r="A828" s="2" t="n">
+        <x:v>3411</x:v>
+      </x:c>
+      <x:c r="B828" s="2" t="str">
+        <x:v>EidolonText331</x:v>
+      </x:c>
+      <x:c r="C828" s="3" t="str">
+        <x:v>학습 단계 수를 직접 입력할 수 있습니다. 빠른 학습은 {0}단계, 기본 학습은 {1}단계입니다. 단계를 줄이면 학습 시간과 품질이 달라질 수 있습니다.</x:v>
+      </x:c>
+      <x:c r="D828" s="3" t="str">
+        <x:v>Enter a training step count. Quick uses {0} steps and Standard uses {1}. Fewer steps change training time and may reduce quality.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="829">
+      <x:c r="A829" s="2" t="n">
+        <x:v>3412</x:v>
+      </x:c>
+      <x:c r="B829" s="2" t="str">
+        <x:v>EidolonText332</x:v>
+      </x:c>
+      <x:c r="C829" s="3" t="str">
+        <x:v>폴더 열기</x:v>
+      </x:c>
+      <x:c r="D829" s="3" t="str">
+        <x:v>Open folder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="830">
+      <x:c r="A830" s="2" t="n">
+        <x:v>3413</x:v>
+      </x:c>
+      <x:c r="B830" s="2" t="str">
+        <x:v>EidolonText333</x:v>
+      </x:c>
+      <x:c r="C830" s="3" t="str">
+        <x:v>폴더로 변경</x:v>
+      </x:c>
+      <x:c r="D830" s="3" t="str">
+        <x:v>Switch to folder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="831">
+      <x:c r="A831" s="2" t="n">
+        <x:v>3414</x:v>
+      </x:c>
+      <x:c r="B831" s="2" t="str">
+        <x:v>EidolonText334</x:v>
+      </x:c>
+      <x:c r="C831" s="3" t="str">
+        <x:v>선택한 폴더와 하위 폴더의 모든 이미지로 학습합니다. 이미지와 같은 이름의 .txt 파일이 있으면 설명으로 사용합니다.</x:v>
+      </x:c>
+      <x:c r="D831" s="3" t="str">
+        <x:v>Train with every image in the selected folder and its subfolders. A .txt file with the same name as an image provides its caption.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="832">
+      <x:c r="A832" s="2" t="n">
+        <x:v>3415</x:v>
+      </x:c>
+      <x:c r="B832" s="2" t="str">
+        <x:v>EidolonText335</x:v>
+      </x:c>
+      <x:c r="C832" s="3" t="str">
+        <x:v>학습 단계 수</x:v>
+      </x:c>
+      <x:c r="D832" s="3" t="str">
+        <x:v>Training steps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="833">
+      <x:c r="A833" s="2" t="n">
+        <x:v>3416</x:v>
+      </x:c>
+      <x:c r="B833" s="2" t="str">
+        <x:v>EidolonText336</x:v>
+      </x:c>
+      <x:c r="C833" s="3" t="str">
+        <x:v>기본 학습</x:v>
+      </x:c>
+      <x:c r="D833" s="3" t="str">
+        <x:v>Standard training</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="834">
+      <x:c r="A834" s="2" t="n">
+        <x:v>3417</x:v>
+      </x:c>
+      <x:c r="B834" s="2" t="str">
+        <x:v>EidolonText337</x:v>
+      </x:c>
+      <x:c r="C834" s="3" t="str">
+        <x:v>이 단어로 LoRA를 학습합니다. 생성 화면에서 이 LoRA를 선택하면 프롬프트에 자동으로 적용됩니다.</x:v>
+      </x:c>
+      <x:c r="D834" s="3" t="str">
+        <x:v>Train this LoRA with this keyword. Selecting this LoRA in Generate automatically applies it to the prompt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="835">
+      <x:c r="A835" s="2" t="n">
+        <x:v>3418</x:v>
+      </x:c>
+      <x:c r="B835" s="2" t="str">
+        <x:v>EidolonText338</x:v>
+      </x:c>
+      <x:c r="C835" s="3" t="str">
+        <x:v>학습 단계 수는 {0}~{1} 사이의 정수로 입력하세요.</x:v>
+      </x:c>
+      <x:c r="D835" s="3" t="str">
+        <x:v>Enter a whole number of training steps between {0} and {1}.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="836">
+      <x:c r="A836" s="2" t="n">
+        <x:v>3419</x:v>
+      </x:c>
+      <x:c r="B836" s="2" t="str">
+        <x:v>EidolonText339</x:v>
+      </x:c>
+      <x:c r="C836" s="3" t="str">
+        <x:v>학습 설정</x:v>
+      </x:c>
+      <x:c r="D836" s="3" t="str">
+        <x:v>Training settings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="837">
+      <x:c r="A837" s="2" t="n">
+        <x:v>3420</x:v>
+      </x:c>
+      <x:c r="B837" s="2" t="str">
+        <x:v>EidolonText340</x:v>
+      </x:c>
+      <x:c r="C837" s="3" t="str">
+        <x:v>자동 적용 트리거: {0}</x:v>
+      </x:c>
+      <x:c r="D837" s="3" t="str">
+        <x:v>Automatic triggers: {0}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="838">
+      <x:c r="A838" s="2" t="n">
+        <x:v>3421</x:v>
+      </x:c>
+      <x:c r="B838" s="2" t="str">
+        <x:v>EidolonText341</x:v>
+      </x:c>
+      <x:c r="C838" s="3" t="str">
+        <x:v>이 모델에 사용할 수 있는 LoRA가 없습니다.</x:v>
+      </x:c>
+      <x:c r="D838" s="3" t="str">
+        <x:v>No LoRAs are available for this model.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="839">
+      <x:c r="A839" s="2" t="n">
+        <x:v>3422</x:v>
+      </x:c>
+      <x:c r="B839" s="2" t="str">
+        <x:v>EidolonText342</x:v>
+      </x:c>
+      <x:c r="C839" s="3" t="str">
+        <x:v>현재 작업이 끝난 뒤 설정을 저장할 수 있습니다.</x:v>
+      </x:c>
+      <x:c r="D839" s="3" t="str">
+        <x:v>Save settings once the current work finishes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>